<commit_message>
gaussblur5x5 intshift code and data
</commit_message>
<xml_diff>
--- a/filter-cases/final_img/5x5/metrics_5x5.xlsx
+++ b/filter-cases/final_img/5x5/metrics_5x5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\fysiko_apth\ptuxiaki\thesis-cases\final_img\5x5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{698D7B2C-4F53-4547-8364-756DC176936C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35352BA4-3298-4E5E-8848-398ADC170D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30132" yWindow="588" windowWidth="23040" windowHeight="11976" xr2:uid="{1A5AD2DC-DE0B-4FFA-AE19-FC07F326EFA1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
   <si>
     <t>output text</t>
   </si>
@@ -821,21 +821,57 @@
       <c r="C9" t="s">
         <v>37</v>
       </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I9">
+        <v>32508</v>
+      </c>
+      <c r="J9">
+        <v>14574</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>68</v>
+      </c>
+      <c r="M9">
+        <v>0.19400000000000001</v>
+      </c>
+      <c r="N9">
+        <v>1485</v>
+      </c>
+      <c r="O9">
+        <v>179224</v>
+      </c>
       <c r="P9">
         <f>N9+($F$2*$E$2)</f>
-        <v>175812</v>
+        <v>177297</v>
       </c>
       <c r="Q9">
-        <f>1000/(T9-M9)</f>
-        <v>76.92307692307692</v>
+        <f>1000/(T9-O9)</f>
+        <v>-5.5800146196383037E-3</v>
       </c>
       <c r="R9">
         <f>U9*Q9</f>
-        <v>76.92307692307692</v>
+        <v>-5.5800146196383037E-3</v>
       </c>
       <c r="S9">
         <f>Q9*10^6/P9</f>
-        <v>437.53029897320386</v>
+        <v>-3.1472696208273712E-2</v>
       </c>
       <c r="T9">
         <v>13</v>
@@ -854,21 +890,57 @@
       <c r="C11" t="s">
         <v>40</v>
       </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>0.49991467595100397</v>
+      </c>
+      <c r="F11">
+        <v>0.70704644918441695</v>
+      </c>
+      <c r="G11">
+        <v>0.99883667465734205</v>
+      </c>
+      <c r="H11">
+        <v>51.141844773077203</v>
+      </c>
+      <c r="I11">
+        <v>4540</v>
+      </c>
+      <c r="J11">
+        <v>12173</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>2.8690000000000002</v>
+      </c>
+      <c r="N11">
+        <v>1479</v>
+      </c>
+      <c r="O11">
+        <v>179218</v>
+      </c>
       <c r="P11">
         <f>N11+($F$2*$E$2)</f>
-        <v>175812</v>
+        <v>177291</v>
       </c>
       <c r="Q11">
         <f>1000/(T11-M11)</f>
-        <v>76.92307692307692</v>
+        <v>98.706939097818577</v>
       </c>
       <c r="R11">
         <f t="shared" ref="R11" si="0">U11*Q11</f>
-        <v>76.92307692307692</v>
+        <v>98.706939097818577</v>
       </c>
       <c r="S11">
         <f>Q11*10^6/P11</f>
-        <v>437.53029897320386</v>
+        <v>556.7509862193715</v>
       </c>
       <c r="T11">
         <v>13</v>

</xml_diff>

<commit_message>
gauss5x5 ieee code and results
</commit_message>
<xml_diff>
--- a/filter-cases/final_img/5x5/metrics_5x5.xlsx
+++ b/filter-cases/final_img/5x5/metrics_5x5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\fysiko_apth\ptuxiaki\thesis-cases\final_img\5x5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35352BA4-3298-4E5E-8848-398ADC170D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A559F514-0057-4985-8CD1-971EB95ADEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30132" yWindow="588" windowWidth="23040" windowHeight="11976" xr2:uid="{1A5AD2DC-DE0B-4FFA-AE19-FC07F326EFA1}"/>
+    <workbookView xWindow="-23280" yWindow="2784" windowWidth="23004" windowHeight="11976" xr2:uid="{1A5AD2DC-DE0B-4FFA-AE19-FC07F326EFA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -959,21 +959,57 @@
       <c r="C12" t="s">
         <v>43</v>
       </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>0.49991467595100397</v>
+      </c>
+      <c r="F12">
+        <v>0.70704644918441695</v>
+      </c>
+      <c r="G12">
+        <v>0.99883667465734205</v>
+      </c>
+      <c r="H12">
+        <v>51.141844773077203</v>
+      </c>
+      <c r="I12">
+        <v>21293</v>
+      </c>
+      <c r="J12">
+        <v>13643</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>44</v>
+      </c>
+      <c r="M12">
+        <v>1.7609999999999999</v>
+      </c>
+      <c r="N12">
+        <v>1485</v>
+      </c>
+      <c r="O12">
+        <v>179224</v>
+      </c>
       <c r="P12">
         <f>N12+($F$2*$E$2)</f>
-        <v>175812</v>
+        <v>177297</v>
       </c>
       <c r="Q12">
         <f>1000/(T12-M12)</f>
-        <v>76.92307692307692</v>
+        <v>88.975887534478147</v>
       </c>
       <c r="R12">
         <f>U12*Q12</f>
-        <v>76.92307692307692</v>
+        <v>88.975887534478147</v>
       </c>
       <c r="S12">
         <f>Q12*10^6/P12</f>
-        <v>437.53029897320386</v>
+        <v>501.84654864142169</v>
       </c>
       <c r="T12">
         <v>13</v>

</xml_diff>